<commit_message>
BE-04 unfrozen: frozen to open (Vatsal, 28 Sep 2026); status changes by commit through data/sq_overrides.json
data/sq_overrides.json holds status changes made after the answer set; scripts/import_sq.py applies them after
reading the answer set and writes each into the row's log (date, from, to, cause, note), so a rewrite keeps them and
the answer text never changes. BE-04 is open, owner Product, no date, the item to follow; the tab lists it with the
open and owed rows (10 now: 221 frozen, 7 open, 3 owed) and shows the log line. The importer now carries the export
stamps across rewrites (it had reset them), and the export places its added columns after the last cell with
content rather than after Excel's empty trailing cells. Export restamped 28 Sep 2026: BE-04 reads "open - to be
decided" and "yes" under "Changed since 26 Sep 2026".
</commit_message>
<xml_diff>
--- a/docs/exports/SQ1_2026_Sep_22nd_Frontend_Technical_Questionaire.xlsx
+++ b/docs/exports/SQ1_2026_Sep_22nd_Frontend_Technical_Questionaire.xlsx
@@ -120,7 +120,7 @@
       </c>
       <c r="I2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Changed since previous export (first export 26 Sep 2026)</t>
+          <t xml:space="preserve">Changed since 26 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -3367,7 +3367,7 @@
       </c>
       <c r="H2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Changed since previous export (first export 26 Sep 2026)</t>
+          <t xml:space="preserve">Changed since 26 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -3612,7 +3612,7 @@
       </c>
       <c r="H2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Changed since previous export (first export 26 Sep 2026)</t>
+          <t xml:space="preserve">Changed since 26 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -3767,7 +3767,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <cols>
     <col min="5" max="5" width="60" customWidth="1"/>
-    <col min="8" max="8" width="44" customWidth="1"/>
+    <col min="6" max="6" width="44" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3803,19 +3803,19 @@
           <t xml:space="preserve">Yesly Comments</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Status</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Board ref</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Status</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">Board ref</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">Changed since previous export (first export 26 Sep 2026)</t>
+          <t xml:space="preserve">Changed since 26 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -3845,7 +3845,7 @@
           <t xml:space="preserve">Accepted as proposed (see FE-02).</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr" s="2">
+      <c r="F3" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">frozen</t>
         </is>
@@ -3877,12 +3877,12 @@
           <t xml:space="preserve">Accepted in principle: the New Architecture on. The exact version is FE-01 (W36).</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">frozen</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
+      <c r="F4" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">frozen</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t xml:space="preserve">W36</t>
         </is>
@@ -3914,12 +3914,12 @@
           <t xml:space="preserve">Accepted as proposed. The version claims in the cell ("default in RN 0.87+", "Node 22.13+", "Kotlin 2.0+") are Spinach's to verify against the pinned versions (W36); HoA does not check them.</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">frozen</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
+      <c r="F5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">frozen</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
         <is>
           <t xml:space="preserve">W36</t>
         </is>
@@ -3951,7 +3951,7 @@
           <t xml:space="preserve">Accepted. Folder and route names follow the board's section letters (FE-11, FE-15), so a screen ID, a route, a folder and an event name all read the same.</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr" s="2">
+      <c r="F6" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">frozen</t>
         </is>
@@ -3983,7 +3983,7 @@
           <t xml:space="preserve">Accepted with FE-76's condition.</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr" s="2">
+      <c r="F7" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">frozen</t>
         </is>
@@ -4015,7 +4015,7 @@
           <t xml:space="preserve">Accepted (FE-20).</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr" s="2">
+      <c r="F8" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">frozen</t>
         </is>
@@ -4252,7 +4252,7 @@
       </c>
       <c r="H2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Changed since previous export (first export 26 Sep 2026)</t>
+          <t xml:space="preserve">Changed since 26 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="H2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Changed since previous export (first export 26 Sep 2026)</t>
+          <t xml:space="preserve">Changed since 26 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -4674,7 +4674,7 @@
       </c>
       <c r="H2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Changed since previous export (first export 26 Sep 2026)</t>
+          <t xml:space="preserve">Changed since 26 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -4936,7 +4936,7 @@
       </c>
       <c r="H2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Changed since previous export (first export 26 Sep 2026)</t>
+          <t xml:space="preserve">Changed since 26 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -5224,7 +5224,7 @@
       </c>
       <c r="H2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Changed since previous export (first export 26 Sep 2026)</t>
+          <t xml:space="preserve">Changed since 26 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -5487,7 +5487,7 @@
       </c>
       <c r="H2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Changed since previous export (first export 26 Sep 2026)</t>
+          <t xml:space="preserve">Changed since 26 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -5712,7 +5712,7 @@
       </c>
       <c r="H2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Changed since previous export (first export 26 Sep 2026)</t>
+          <t xml:space="preserve">Changed since 26 Sep 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Export carries the board comments: the latest comment per row appended to the Yesly Comments cell
scripts/export_sq.py reads data/board_entries.json (page spinach_questions, field comment; the latest non-empty row
per question) and appends it to the row's exported cell as "Update, <first name>, <date>: <text>"; the answer text is
unchanged. A comment newer than the last stamp counts as a change for the stamp and the "Changed since" marks. Board
pulled 28 Sep 2026 (188 rows): 10 rows carry a comment, all Vatsal's of 28 Sep 2026; the pull also refreshes the
board-fed blobs on the wireframes and admin pages. The tab says that comments carry once the board is pulled and
the site rebuilt (scripts/pull_board.py, then scripts/build_site.py).
</commit_message>
<xml_diff>
--- a/docs/exports/SQ1_2026_Sep_22nd_Frontend_Technical_Questionaire.xlsx
+++ b/docs/exports/SQ1_2026_Sep_22nd_Frontend_Technical_Questionaire.xlsx
@@ -152,7 +152,8 @@
       </c>
       <c r="F3" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">to be verified: the exact Expo SDK and React Native versions, pinned by Spinach before development starts and stated in the project plan. The two supplementary sheets give two different floors (0.76+ on Foundation row 2, 0.87+ on row 3); one pair of numbers, please. HoA confirms on receipt.</t>
+          <t xml:space="preserve">to be verified: the exact Expo SDK and React Native versions, pinned by Spinach before development starts and stated in the project plan. The two supplementary sheets give two different floors (0.76+ on Foundation row 2, 0.87+ on row 3); one pair of numbers, please. HoA confirms on receipt.
+Update, Vatsal, 28 Sep 2026: go as per Spinach's proposal</t>
         </is>
       </c>
       <c r="G3" t="inlineStr" s="2">
@@ -163,6 +164,11 @@
       <c r="H3" t="inlineStr">
         <is>
           <t xml:space="preserve">W36</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
     </row>
@@ -794,7 +800,8 @@
       </c>
       <c r="F19" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">to be verified: there is no Figma yet. Spinach owns visual design and produces it after the frozen wireframes. Until an approved visual design exists, Wireframes v0.2 on the board is the source of truth for structure, fields, tags, states and events. The Figma file and its version are recorded on X00 when they exist.</t>
+          <t xml:space="preserve">to be verified: there is no Figma yet. Spinach owns visual design and produces it after the frozen wireframes. Until an approved visual design exists, Wireframes v0.2 on the board is the source of truth for structure, fields, tags, states and events. The Figma file and its version are recorded on X00 when they exist.
+Update, Vatsal, 28 Sep 2026: Spinach to give Figma and apply</t>
         </is>
       </c>
       <c r="G19" t="inlineStr" s="2">
@@ -805,6 +812,11 @@
       <c r="H19" t="inlineStr">
         <is>
           <t xml:space="preserve">X00, W22</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
     </row>
@@ -3053,7 +3065,8 @@
       </c>
       <c r="F76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">to be decided: the iOS bundle ID and the Android package name, the reverse of HoA's domain once the domain is confirmed (W35).</t>
+          <t xml:space="preserve">to be decided: the iOS bundle ID and the Android package name, the reverse of HoA's domain once the domain is confirmed (W35).
+Update, Vatsal, 28 Sep 2026: we will revert with this week Thursday</t>
         </is>
       </c>
       <c r="G76" t="inlineStr" s="2">
@@ -3064,6 +3077,11 @@
       <c r="H76" t="inlineStr">
         <is>
           <t xml:space="preserve">W35</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
     </row>
@@ -3095,7 +3113,8 @@
       </c>
       <c r="F77" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">to be decided: the Apple Developer and Google Play Console accounts in HoA's legal name; the registration is in, so they can be opened now (W35). The financial-app declarations and the listing text follow (W06, Compliance).</t>
+          <t xml:space="preserve">to be decided: the Apple Developer and Google Play Console accounts in HoA's legal name; the registration is in, so they can be opened now (W35). The financial-app declarations and the listing text follow (W06, Compliance).
+Update, Vatsal, 28 Sep 2026: With Raafiya to open the account - will be ready after next 2 weeks</t>
         </is>
       </c>
       <c r="G77" t="inlineStr" s="2">
@@ -3106,6 +3125,11 @@
       <c r="H77" t="inlineStr">
         <is>
           <t xml:space="preserve">W35, W06</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
     </row>
@@ -3211,7 +3235,8 @@
       </c>
       <c r="F80" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">to be decided: the store listing copy (owner: Copy) and the financial-app declarations (owner: Compliance, W06). Spinach handles the technical submission, as proposed.</t>
+          <t xml:space="preserve">to be decided: the store listing copy (owner: Copy) and the financial-app declarations (owner: Compliance, W06). Spinach handles the technical submission, as proposed.
+Update, Vatsal, 28 Sep 2026: With Raafiya to open the account - will be ready after next 6 weeks</t>
         </is>
       </c>
       <c r="G80" t="inlineStr" s="2">
@@ -3222,6 +3247,11 @@
       <c r="H80" t="inlineStr">
         <is>
           <t xml:space="preserve">W06</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
     </row>

</xml_diff>